<commit_message>
Web Application & MCP Update
</commit_message>
<xml_diff>
--- a/load_and_merge_scripts/data/model.xlsx
+++ b/load_and_merge_scripts/data/model.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R67ec631187e64436"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="2" r:id="R4cb03bb1a7984d84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelScope" sheetId="3" r:id="R68677c4e1980449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_README" sheetId="1" r:id="R998d46370e7f4b83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="2" r:id="Ra26ce0f1d49e43ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelScope" sheetId="3" r:id="R5745c829ecc54c3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -665,13 +665,13 @@
         <x:v>model_description</x:v>
       </x:c>
       <x:c r="D1" s="47" t="str">
-        <x:v>silver_model_naming_template</x:v>
+        <x:v>silver_model_naming_instructions</x:v>
       </x:c>
       <x:c r="E1" s="47" t="str">
         <x:v>silver_model_audit_columns_template</x:v>
       </x:c>
       <x:c r="F1" s="47" t="str">
-        <x:v>gold_model_naming_template</x:v>
+        <x:v>gold_model_naming_instructions</x:v>
       </x:c>
       <x:c r="G1" s="47" t="str">
         <x:v>gold_model_technical_columns_template</x:v>

</xml_diff>